<commit_message>
Switch to the church's nine book categories
</commit_message>
<xml_diff>
--- a/docs/templates/book-donation-template.xlsx
+++ b/docs/templates/book-donation-template.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Christian living</t>
+          <t>Christian Living</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -536,7 +536,6 @@
       <c r="H2" t="n">
         <v>2001</v>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -562,7 +561,6 @@
           <t>New</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>Zonderkidz</t>
@@ -580,7 +578,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Category" error="Pick a category from the list." type="list">
-      <formula1>=Lists!$A$2:$A$11</formula1>
+      <formula1>=Lists!$A$2:$A$10</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$C$2:$C$4</formula1>
@@ -600,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -613,7 +611,6 @@
           <t>Allowed categories</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
       <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Allowed conditions</t>
@@ -623,7 +620,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bible &amp; study</t>
+          <t>Bible Study &amp; Doctrine</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -635,7 +632,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Devotional</t>
+          <t>Biography &amp; Testimony</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -647,7 +644,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Christian living</t>
+          <t>Christian Living</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -659,52 +656,47 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Theology</t>
+          <t>Church &amp; Ministry</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Biography</t>
+          <t>Evangelism &amp; Missions</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Children</t>
+          <t>Leadership</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Classics</t>
+          <t>Marriage, Family &amp; Relationships</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Apologetics</t>
+          <t>Prayer &amp; Worship</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hymnals &amp; music</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-    </row>
+          <t>Society &amp; Culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>